<commit_message>
Add assets, scripts, and content updates
- Update starter kit colour collection xlsx and price list CSV
- Replace premium-builder.jpg with updated image
- Add PPWR packaging compliance declaration webp
- Add Gelitup Ambassador Letter docx
- Add certificate utility scripts (blur, crop, grid, date verify)
- Add Reunion creative brief (PDF + HTML)
- Add deno.lock

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Starter-kit-colour-collection-.xlsx
+++ b/Starter-kit-colour-collection-.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Leeukopf-Website-Official\gelitup-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF54D52F-6C84-4839-BCE4-1CFA4E7CC3D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B911B11-ED6A-496C-BDD1-7D5BDE721FBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{4FA4370A-4E17-4679-8040-16958C1E37CA}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{4FA4370A-4E17-4679-8040-16958C1E37CA}"/>
   </bookViews>
   <sheets>
     <sheet name="Beginner Colour Kit" sheetId="8" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="145">
   <si>
     <t>Superbond without Acid</t>
   </si>
@@ -437,24 +437,9 @@
     <t>MultiMix Synthogel 60gr Glitter White -HTF</t>
   </si>
   <si>
-    <t>DUAL FORMS ALMOND</t>
-  </si>
-  <si>
     <t>DUAL FORMS BALLERINA</t>
   </si>
   <si>
-    <t>DUAL FORMS LONG ALMOND</t>
-  </si>
-  <si>
-    <t>DUAL FORMS MODERN SQUARE</t>
-  </si>
-  <si>
-    <t>DUAL FORMS RUSSIAN ALMOND</t>
-  </si>
-  <si>
-    <t>DUAL FORMS SQUARE</t>
-  </si>
-  <si>
     <t>DUAL FORMS SQUOVAL</t>
   </si>
   <si>
@@ -483,6 +468,12 @@
   </si>
   <si>
     <t>74 Sailor She -HTF</t>
+  </si>
+  <si>
+    <t>NAIL EXTENSION DUAL FORMS RUSSIAN ALMOND</t>
+  </si>
+  <si>
+    <t>NAIL EXTENSION DUAL FORMS SQUARE</t>
   </si>
 </sst>
 </file>
@@ -491,7 +482,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="_([$€-2]\ * #,##0.00_);_([$€-2]\ * \(#,##0.00\);_([$€-2]\ * &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="169" formatCode="[$€-2]\ #,##0.00;[Red]\-[$€-2]\ #,##0.00"/>
+    <numFmt numFmtId="165" formatCode="[$€-2]\ #,##0.00;[Red]\-[$€-2]\ #,##0.00"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -577,7 +568,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -591,14 +582,13 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -942,27 +932,27 @@
     </row>
     <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="10" t="s">
-        <v>139</v>
+      <c r="A7" s="9" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="10" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="B9">
         <v>59.45</v>
@@ -1004,38 +994,38 @@
       </c>
     </row>
     <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
-        <v>144</v>
+      <c r="A5" s="3" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1445,7 +1435,7 @@
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A93" s="3" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.3">
@@ -2226,7 +2216,397 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDAD115B-50CC-4FA4-B8CB-5A2628C1856B}">
-  <dimension ref="A1:B107"/>
+  <dimension ref="A1:B104"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="43.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B5" s="3"/>
+    </row>
+    <row r="6" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B6" s="3"/>
+    </row>
+    <row r="7" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>143</v>
+      </c>
+      <c r="B7" s="3"/>
+    </row>
+    <row r="8" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>144</v>
+      </c>
+      <c r="B8" s="3"/>
+    </row>
+    <row r="9" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B9" s="3"/>
+    </row>
+    <row r="10" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B10" s="3"/>
+    </row>
+    <row r="11" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B11" s="3"/>
+    </row>
+    <row r="12" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B12" s="3"/>
+    </row>
+    <row r="13" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="B13" s="3"/>
+    </row>
+    <row r="14" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" s="3" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="3" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="B25" s="11">
+        <v>53.95</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" s="3" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" s="3"/>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" s="3"/>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" s="3"/>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" s="3"/>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" s="3"/>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" s="3"/>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A33" s="3"/>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A34" s="3"/>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A35" s="3"/>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A36" s="3"/>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A37" s="3"/>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A38" s="3"/>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A39" s="3"/>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A40" s="3"/>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A41" s="3"/>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A42" s="3"/>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A43" s="3"/>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A44" s="2"/>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A45" s="3"/>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A46" s="3"/>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A47" s="3"/>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A48" s="3"/>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A49" s="3"/>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A50" s="3"/>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A51" s="3"/>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A52" s="3"/>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A53" s="3"/>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A54" s="3"/>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A55" s="3"/>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A56" s="3"/>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A57" s="3"/>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A58" s="3"/>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A59" s="3"/>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A60" s="3"/>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A61" s="3"/>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A62" s="3"/>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A63" s="3"/>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A64" s="3"/>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A65" s="3"/>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A66" s="3"/>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A67" s="3"/>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A68" s="3"/>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A69" s="3"/>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A70" s="3"/>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A71" s="3"/>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A72" s="3"/>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A73" s="3"/>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A74" s="3"/>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A75" s="3"/>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A76" s="3"/>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A77" s="3"/>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A78" s="3"/>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A79" s="3"/>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A80" s="3"/>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A81" s="2"/>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A82" s="3"/>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A83" s="3"/>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A84" s="3"/>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A85" s="3"/>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A86" s="3"/>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A87" s="3"/>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A88" s="3"/>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A89" s="3"/>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A90" s="3"/>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A91" s="3"/>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A92" s="3"/>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A93" s="3"/>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A94" s="3"/>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A95" s="3"/>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A96" s="3"/>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A97" s="3"/>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A98" s="3"/>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A99" s="3"/>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A100" s="3"/>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A101" s="3"/>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A102" s="3"/>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A103" s="3"/>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A104" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFFA9937-09D1-42A6-B54A-C2ADCA4BDD57}">
+  <dimension ref="A1:B116"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="38.33203125" bestFit="1" customWidth="1"/>
@@ -2238,415 +2618,6 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="B6" s="3"/>
-    </row>
-    <row r="7" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="B7" s="3"/>
-    </row>
-    <row r="8" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="B8" s="3"/>
-    </row>
-    <row r="9" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="B9" s="3"/>
-    </row>
-    <row r="10" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="B10" s="3"/>
-    </row>
-    <row r="11" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="B11" s="3"/>
-    </row>
-    <row r="12" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="B12" s="3"/>
-    </row>
-    <row r="13" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="B13" s="3"/>
-    </row>
-    <row r="14" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="B14" s="3"/>
-    </row>
-    <row r="15" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B15" s="3"/>
-    </row>
-    <row r="16" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="B16" s="3"/>
-    </row>
-    <row r="17" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="B17" s="3"/>
-    </row>
-    <row r="18" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="B18" s="3"/>
-    </row>
-    <row r="19" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="3" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="3" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A21" s="3" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A22" s="3" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A23" s="3" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" s="3" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A25" s="3" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A26" s="3" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27" s="3" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A28" s="3" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A29" s="3" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A30" s="3"/>
-      <c r="B30" s="12">
-        <v>53.95</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A31" s="3"/>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A32" s="3"/>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A33" s="3"/>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A34" s="3"/>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A35" s="3"/>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A36" s="3"/>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A37" s="3"/>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A38" s="3"/>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A39" s="3"/>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A40" s="3"/>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A41" s="3"/>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A42" s="3"/>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A43" s="3"/>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A44" s="3"/>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A45" s="3"/>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A46" s="3"/>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A47" s="2"/>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A48" s="3"/>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A49" s="3"/>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A50" s="3"/>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A51" s="3"/>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A52" s="3"/>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A53" s="3"/>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A54" s="3"/>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A55" s="3"/>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A56" s="3"/>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A57" s="3"/>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A58" s="3"/>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A59" s="3"/>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A60" s="3"/>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A61" s="3"/>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A62" s="3"/>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A63" s="3"/>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A64" s="3"/>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A65" s="3"/>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A66" s="3"/>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A67" s="3"/>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A68" s="3"/>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A69" s="3"/>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A70" s="3"/>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A71" s="3"/>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A72" s="3"/>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A73" s="3"/>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A74" s="3"/>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A75" s="3"/>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A76" s="3"/>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A77" s="3"/>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A78" s="3"/>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A79" s="3"/>
-    </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A80" s="3"/>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A81" s="3"/>
-    </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A82" s="3"/>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A83" s="3"/>
-    </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A84" s="2"/>
-    </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A85" s="3"/>
-    </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A86" s="3"/>
-    </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A87" s="3"/>
-    </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A88" s="3"/>
-    </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A89" s="3"/>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A90" s="3"/>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A91" s="3"/>
-    </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A92" s="3"/>
-    </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A93" s="3"/>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A94" s="3"/>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A95" s="3"/>
-    </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A96" s="3"/>
-    </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A97" s="3"/>
-    </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A98" s="3"/>
-    </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A99" s="3"/>
-    </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A100" s="3"/>
-    </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A101" s="3"/>
-    </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A102" s="3"/>
-    </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A103" s="3"/>
-    </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A104" s="3"/>
-    </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A105" s="3"/>
-    </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A106" s="3"/>
-    </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A107" s="3"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFFA9937-09D1-42A6-B54A-C2ADCA4BDD57}">
-  <dimension ref="A1:B119"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="38.33203125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B1" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
@@ -2661,597 +2632,578 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>132</v>
       </c>
+      <c r="B5" s="3"/>
     </row>
     <row r="6" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
-        <v>133</v>
+      <c r="A6" t="s">
+        <v>143</v>
       </c>
       <c r="B6" s="3"/>
     </row>
     <row r="7" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
-        <v>134</v>
+      <c r="A7" t="s">
+        <v>144</v>
       </c>
       <c r="B7" s="3"/>
     </row>
     <row r="8" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B8" s="3"/>
     </row>
     <row r="9" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
-        <v>136</v>
+      <c r="A9" s="6" t="s">
+        <v>115</v>
       </c>
       <c r="B9" s="3"/>
     </row>
     <row r="10" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
-        <v>137</v>
+      <c r="A10" s="6" t="s">
+        <v>101</v>
       </c>
       <c r="B10" s="3"/>
     </row>
     <row r="11" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="3" t="s">
-        <v>138</v>
+      <c r="A11" s="6" t="s">
+        <v>99</v>
       </c>
       <c r="B11" s="3"/>
     </row>
     <row r="12" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="B12" s="3"/>
     </row>
     <row r="13" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="6" t="s">
-        <v>101</v>
+      <c r="A13" s="3" t="s">
+        <v>139</v>
       </c>
       <c r="B13" s="3"/>
     </row>
     <row r="14" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="6" t="s">
-        <v>99</v>
+      <c r="A14" s="3" t="s">
+        <v>140</v>
       </c>
       <c r="B14" s="3"/>
     </row>
     <row r="15" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="6" t="s">
-        <v>100</v>
+      <c r="A15" s="1" t="s">
+        <v>134</v>
       </c>
       <c r="B15" s="3"/>
     </row>
     <row r="16" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="B16" s="3"/>
+        <v>138</v>
+      </c>
     </row>
     <row r="17" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="B17" s="3"/>
-    </row>
-    <row r="18" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="B18" s="3"/>
-    </row>
-    <row r="19" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="B19" s="3"/>
-    </row>
-    <row r="20" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="B20" s="3"/>
-    </row>
-    <row r="21" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
-        <v>140</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
-        <v>3</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
-        <v>4</v>
+        <v>63</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
-        <v>5</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
-        <v>63</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="B27" s="4"/>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="B32" s="4"/>
+        <v>66</v>
+      </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" s="3" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" s="3" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53" s="3" t="s">
-        <v>89</v>
+        <v>23</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" s="3" t="s">
-        <v>90</v>
+        <v>24</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A55" s="3" t="s">
-        <v>91</v>
+      <c r="A55" s="2" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A56" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A58" s="2" t="s">
-        <v>61</v>
+      <c r="A58" s="3" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A59" s="3" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A60" s="3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A61" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A62" s="3" t="s">
-        <v>28</v>
+        <v>6</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A63" s="3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A64" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A65" s="3" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A66" s="3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A67" s="3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A68" s="3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A69" s="3" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A70" s="3" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A71" s="3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A72" s="3" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A73" s="3" t="s">
-        <v>38</v>
+        <v>7</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A74" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A75" s="3" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A76" s="3" t="s">
-        <v>7</v>
+        <v>43</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A77" s="3" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A78" s="3" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A79" s="3" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A80" s="3" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A81" s="3" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A82" s="3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A83" s="3" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A84" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A85" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A86" s="3" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A87" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A88" s="3" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A89" s="3" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A90" s="3" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A91" s="3" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A92" s="3" t="s">
-        <v>56</v>
+      <c r="A92" s="2" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A93" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A94" s="3" t="s">
-        <v>58</v>
+        <v>8</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A95" s="2" t="s">
-        <v>60</v>
+      <c r="A95" s="3" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A96" s="3" t="s">
-        <v>59</v>
+        <v>10</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A97" s="3" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A98" s="3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A99" s="3" t="s">
-        <v>10</v>
+        <v>142</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A100" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A101" s="3" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A102" s="3" t="s">
-        <v>147</v>
+        <v>13</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A103" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A104" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A105" s="3" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A106" s="3" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A107" s="3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A108" s="3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A109" s="3" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A110" s="3" t="s">
-        <v>20</v>
+        <v>92</v>
       </c>
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A111" s="3" t="s">
-        <v>21</v>
+        <v>93</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A112" s="3" t="s">
-        <v>22</v>
+        <v>94</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A113" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
+      </c>
+      <c r="B113">
+        <v>167.45</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A114" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A115" s="3" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A116" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A117" s="3" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A118" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B118">
-        <v>167.45</v>
-      </c>
-    </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A119" s="3" t="s">
         <v>98</v>
       </c>
     </row>

</xml_diff>